<commit_message>
fix: refine premium template chart layout and transparent backgrounds
</commit_message>
<xml_diff>
--- a/templates/PLANQLY_PREMIUM_TEMPLATE.xlsx
+++ b/templates/PLANQLY_PREMIUM_TEMPLATE.xlsx
@@ -762,6 +762,12 @@
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <spPr>
+      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+      </a:ln>
+    </spPr>
     <title>
       <tx>
         <rich>
@@ -778,6 +784,12 @@
       </tx>
     </title>
     <plotArea>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
       <pieChart>
         <varyColors val="1"/>
         <ser>
@@ -863,6 +875,12 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -874,6 +892,12 @@
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <spPr>
+      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+      </a:ln>
+    </spPr>
     <title>
       <tx>
         <rich>
@@ -890,6 +914,12 @@
       </tx>
     </title>
     <plotArea>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -977,6 +1007,12 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -988,6 +1024,12 @@
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <spPr>
+      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+      </a:ln>
+    </spPr>
     <title>
       <tx>
         <rich>
@@ -1004,6 +1046,12 @@
       </tx>
     </title>
     <plotArea>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
       <areaChart>
         <grouping val="standard"/>
         <ser>
@@ -1059,6 +1107,12 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1070,6 +1124,12 @@
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <spPr>
+      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+      </a:ln>
+    </spPr>
     <title>
       <tx>
         <rich>
@@ -1086,6 +1146,12 @@
       </tx>
     </title>
     <plotArea>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -1162,6 +1228,12 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1173,6 +1245,12 @@
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <spPr>
+      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+      </a:ln>
+    </spPr>
     <title>
       <tx>
         <rich>
@@ -1189,6 +1267,12 @@
       </tx>
     </title>
     <plotArea>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
       <lineChart>
         <grouping val="standard"/>
         <ser>
@@ -1279,6 +1363,12 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1290,6 +1380,12 @@
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <spPr>
+      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+      </a:ln>
+    </spPr>
     <title>
       <tx>
         <rich>
@@ -1306,6 +1402,12 @@
       </tx>
     </title>
     <plotArea>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
       <pieChart>
         <varyColors val="1"/>
         <ser>
@@ -1423,6 +1525,12 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
+      <spPr>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+        </a:ln>
+      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1436,10 +1544,10 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3600000" cy="3960000"/>
+    <ext cx="3000000" cy="3000000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1458,10 +1566,10 @@
     <from>
       <col>13</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3960000"/>
+    <ext cx="3000000" cy="3000000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1478,12 +1586,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>20</col>
+      <col>19</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="3960000"/>
+    <ext cx="3000000" cy="3000000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1502,10 +1610,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>57</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="3600000"/>
+    <ext cx="4200000" cy="3200000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1522,12 +1630,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
-      <row>57</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3600000"/>
+    <ext cx="4200000" cy="3200000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="5" name="Chart 5"/>
@@ -1544,12 +1652,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>16</col>
+      <col>15</col>
       <colOff>0</colOff>
-      <row>57</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3600000"/>
+    <ext cx="4200000" cy="3200000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="6" name="Chart 6"/>

</xml_diff>

<commit_message>
fix: restore visible charts and improve spreadsheet readability
</commit_message>
<xml_diff>
--- a/templates/PLANQLY_PREMIUM_TEMPLATE.xlsx
+++ b/templates/PLANQLY_PREMIUM_TEMPLATE.xlsx
@@ -1220,14 +1220,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
-    <spPr>
-      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:noFill/>
-      </a:ln>
-    </spPr>
     <title>
       <tx>
         <rich>
@@ -1244,12 +1237,6 @@
       </tx>
     </title>
     <plotArea>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
       <pieChart>
         <varyColors val="1"/>
         <ser>
@@ -1316,9 +1303,9 @@
             </spPr>
           </dPt>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$AN$100:$AN$104</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1335,12 +1322,6 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1350,14 +1331,7 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
-    <spPr>
-      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:noFill/>
-      </a:ln>
-    </spPr>
     <title>
       <tx>
         <rich>
@@ -1374,12 +1348,6 @@
       </tx>
     </title>
     <plotArea>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -1400,9 +1368,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$AP$100:$AP$104</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1427,9 +1395,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$AP$100:$AP$104</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1467,12 +1435,6 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1482,14 +1444,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
-    <spPr>
-      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:noFill/>
-      </a:ln>
-    </spPr>
     <title>
       <tx>
         <rich>
@@ -1506,12 +1461,6 @@
       </tx>
     </title>
     <plotArea>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
       <areaChart>
         <grouping val="standard"/>
         <ser>
@@ -1529,9 +1478,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$AT$100:$AT$113</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1567,12 +1516,6 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1582,14 +1525,7 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
-    <spPr>
-      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:noFill/>
-      </a:ln>
-    </spPr>
     <title>
       <tx>
         <rich>
@@ -1606,12 +1542,6 @@
       </tx>
     </title>
     <plotArea>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
@@ -1649,9 +1579,9 @@
             </spPr>
           </dPt>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$AZ$100:$AZ$101</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1688,12 +1618,6 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1703,14 +1627,7 @@
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
-    <spPr>
-      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:noFill/>
-      </a:ln>
-    </spPr>
     <title>
       <tx>
         <rich>
@@ -1727,12 +1644,6 @@
       </tx>
     </title>
     <plotArea>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
       <lineChart>
         <grouping val="standard"/>
         <ser>
@@ -1755,9 +1666,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$BC$100:$BC$129</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1785,9 +1696,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$BC$100:$BC$129</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1823,12 +1734,6 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1838,14 +1743,7 @@
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
-    <spPr>
-      <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-      <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:noFill/>
-      </a:ln>
-    </spPr>
     <title>
       <tx>
         <rich>
@@ -1862,12 +1760,6 @@
       </tx>
     </title>
     <plotArea>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
       <pieChart>
         <varyColors val="1"/>
         <ser>
@@ -1967,9 +1859,9 @@
             </spPr>
           </dPt>
           <cat>
-            <numRef>
+            <strRef>
               <f>'PLANQLY Budget'!$AW$100:$AW$107</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1985,12 +1877,6 @@
     </plotArea>
     <legend>
       <legendPos val="r"/>
-      <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-        </a:ln>
-      </spPr>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>

</xml_diff>

<commit_message>
fix: unfreeze spreadsheet view and restore stable premium template
</commit_message>
<xml_diff>
--- a/templates/PLANQLY_PREMIUM_TEMPLATE.xlsx
+++ b/templates/PLANQLY_PREMIUM_TEMPLATE.xlsx
@@ -1303,9 +1303,9 @@
             </spPr>
           </dPt>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$AN$100:$AN$104</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1368,9 +1368,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$AP$100:$AP$104</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1395,9 +1395,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$AP$100:$AP$104</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1478,9 +1478,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$AT$100:$AT$113</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1579,9 +1579,9 @@
             </spPr>
           </dPt>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$AZ$100:$AZ$101</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1666,9 +1666,9 @@
             </spPr>
           </marker>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$BC$100:$BC$129</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1696,9 +1696,9 @@
             </spPr>
           </marker>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$BC$100:$BC$129</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1859,9 +1859,9 @@
             </spPr>
           </dPt>
           <cat>
-            <strRef>
+            <numRef>
               <f>'PLANQLY Budget'!$AW$100:$AW$107</f>
-            </strRef>
+            </numRef>
           </cat>
           <val>
             <numRef>
@@ -1886,19 +1886,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="twoCell">
+  <oneCellAnchor>
     <from>
       <col>7</col>
       <colOff>0</colOff>
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </to>
+    <ext cx="3600000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1912,20 +1907,15 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="twoCell">
+  </oneCellAnchor>
+  <oneCellAnchor>
     <from>
       <col>13</col>
       <colOff>0</colOff>
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>20</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </to>
+    <ext cx="5040000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1939,20 +1929,15 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="twoCell">
+  </oneCellAnchor>
+  <oneCellAnchor>
     <from>
       <col>20</col>
       <colOff>0</colOff>
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>26</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </to>
+    <ext cx="5760000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1966,20 +1951,15 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="twoCell">
+  </oneCellAnchor>
+  <oneCellAnchor>
     <from>
       <col>1</col>
       <colOff>0</colOff>
       <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>76</row>
-      <rowOff>0</rowOff>
-    </to>
+    <ext cx="4320000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1993,20 +1973,15 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="twoCell">
+  </oneCellAnchor>
+  <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>17</col>
-      <colOff>0</colOff>
-      <row>76</row>
-      <rowOff>0</rowOff>
-    </to>
+    <ext cx="7200000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="5" name="Chart 5"/>
@@ -2020,20 +1995,15 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="twoCell">
+  </oneCellAnchor>
+  <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>57</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>26</col>
-      <colOff>0</colOff>
-      <row>76</row>
-      <rowOff>0</rowOff>
-    </to>
+    <ext cx="5040000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="6" name="Chart 6"/>
@@ -2047,7 +2017,7 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 

</xml_diff>